<commit_message>
logs: nifty precision signals 2026-09-15
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL336"/>
+  <dimension ref="A1:AL338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40868,12 +40868,252 @@
       <c r="AF336" t="n">
         <v>12.29</v>
       </c>
-      <c r="AG336" t="inlineStr"/>
-      <c r="AH336" t="inlineStr"/>
-      <c r="AI336" t="inlineStr"/>
-      <c r="AJ336" t="inlineStr"/>
-      <c r="AK336" t="inlineStr"/>
-      <c r="AL336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D337" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>23200</v>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G337" t="n">
+        <v>23218.4</v>
+      </c>
+      <c r="H337" t="n">
+        <v>85</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K337" t="n">
+        <v>6</v>
+      </c>
+      <c r="L337" t="n">
+        <v>23225.1</v>
+      </c>
+      <c r="M337" t="n">
+        <v>23252.3</v>
+      </c>
+      <c r="N337" t="n">
+        <v>23218.7</v>
+      </c>
+      <c r="O337" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q337" t="n">
+        <v>23588.3</v>
+      </c>
+      <c r="R337" t="n">
+        <v>23452.1</v>
+      </c>
+      <c r="S337" t="n">
+        <v>23447.9</v>
+      </c>
+      <c r="T337" t="n">
+        <v>23232.2</v>
+      </c>
+      <c r="U337" t="n">
+        <v>23378.8</v>
+      </c>
+      <c r="V337" t="n">
+        <v>23340.1</v>
+      </c>
+      <c r="W337" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X337" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y337" t="n">
+        <v>23288.1</v>
+      </c>
+      <c r="Z337" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AA337" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB337" t="n">
+        <v>23258.4</v>
+      </c>
+      <c r="AC337" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD337" t="n">
+        <v>23098.4</v>
+      </c>
+      <c r="AE337" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF337" t="n">
+        <v>13.26</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>23150</v>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G338" t="n">
+        <v>23172.3</v>
+      </c>
+      <c r="H338" t="n">
+        <v>85</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K338" t="n">
+        <v>6</v>
+      </c>
+      <c r="L338" t="n">
+        <v>23187.6</v>
+      </c>
+      <c r="M338" t="n">
+        <v>23218.2</v>
+      </c>
+      <c r="N338" t="n">
+        <v>23178</v>
+      </c>
+      <c r="O338" t="n">
+        <v>27</v>
+      </c>
+      <c r="P338" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q338" t="n">
+        <v>23588.3</v>
+      </c>
+      <c r="R338" t="n">
+        <v>23452.1</v>
+      </c>
+      <c r="S338" t="n">
+        <v>23447.9</v>
+      </c>
+      <c r="T338" t="n">
+        <v>23232.2</v>
+      </c>
+      <c r="U338" t="n">
+        <v>23378.8</v>
+      </c>
+      <c r="V338" t="n">
+        <v>23340.1</v>
+      </c>
+      <c r="W338" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X338" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y338" t="n">
+        <v>23255.3</v>
+      </c>
+      <c r="Z338" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="AA338" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB338" t="n">
+        <v>23212.3</v>
+      </c>
+      <c r="AC338" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD338" t="n">
+        <v>23052.3</v>
+      </c>
+      <c r="AE338" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF338" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="AG338" t="inlineStr"/>
+      <c r="AH338" t="inlineStr"/>
+      <c r="AI338" t="inlineStr"/>
+      <c r="AJ338" t="inlineStr"/>
+      <c r="AK338" t="inlineStr"/>
+      <c r="AL338" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-18
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL338"/>
+  <dimension ref="A1:AL341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41108,12 +41108,372 @@
       <c r="AF338" t="n">
         <v>13.46</v>
       </c>
-      <c r="AG338" t="inlineStr"/>
-      <c r="AH338" t="inlineStr"/>
-      <c r="AI338" t="inlineStr"/>
-      <c r="AJ338" t="inlineStr"/>
-      <c r="AK338" t="inlineStr"/>
-      <c r="AL338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>23350</v>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G339" t="n">
+        <v>23352.9</v>
+      </c>
+      <c r="H339" t="n">
+        <v>81</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K339" t="n">
+        <v>6</v>
+      </c>
+      <c r="L339" t="n">
+        <v>23339.2</v>
+      </c>
+      <c r="M339" t="n">
+        <v>23331.1</v>
+      </c>
+      <c r="N339" t="n">
+        <v>23352.1</v>
+      </c>
+      <c r="O339" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="P339" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q339" t="n">
+        <v>23359.3</v>
+      </c>
+      <c r="R339" t="n">
+        <v>23292.1</v>
+      </c>
+      <c r="S339" t="n">
+        <v>23363.2</v>
+      </c>
+      <c r="T339" t="n">
+        <v>23195.1</v>
+      </c>
+      <c r="U339" t="n">
+        <v>23279.2</v>
+      </c>
+      <c r="V339" t="n">
+        <v>23273.4</v>
+      </c>
+      <c r="W339" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X339" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y339" t="n">
+        <v>23343.6</v>
+      </c>
+      <c r="Z339" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AA339" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB339" t="n">
+        <v>23312.9</v>
+      </c>
+      <c r="AC339" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD339" t="n">
+        <v>23472.9</v>
+      </c>
+      <c r="AE339" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF339" t="n">
+        <v>11.51</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>74600</v>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G340" t="n">
+        <v>74560.60000000001</v>
+      </c>
+      <c r="H340" t="n">
+        <v>81</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K340" t="n">
+        <v>6</v>
+      </c>
+      <c r="L340" t="n">
+        <v>74531.7</v>
+      </c>
+      <c r="M340" t="n">
+        <v>74519</v>
+      </c>
+      <c r="N340" t="n">
+        <v>74548.60000000001</v>
+      </c>
+      <c r="O340" t="n">
+        <v>60</v>
+      </c>
+      <c r="P340" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q340" t="n">
+        <v>74591.2</v>
+      </c>
+      <c r="R340" t="n">
+        <v>74399.3</v>
+      </c>
+      <c r="S340" t="n">
+        <v>74676.3</v>
+      </c>
+      <c r="T340" t="n">
+        <v>74182.60000000001</v>
+      </c>
+      <c r="U340" t="n">
+        <v>74429.5</v>
+      </c>
+      <c r="V340" t="n">
+        <v>74352.89999999999</v>
+      </c>
+      <c r="W340" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X340" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y340" t="n">
+        <v>74545.89999999999</v>
+      </c>
+      <c r="Z340" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="AA340" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB340" t="n">
+        <v>74360.60000000001</v>
+      </c>
+      <c r="AC340" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD340" t="n">
+        <v>75160.60000000001</v>
+      </c>
+      <c r="AE340" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF340" t="n">
+        <v>11.51</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>23350</v>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G341" t="n">
+        <v>23369.4</v>
+      </c>
+      <c r="H341" t="n">
+        <v>88</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K341" t="n">
+        <v>7</v>
+      </c>
+      <c r="L341" t="n">
+        <v>23359.6</v>
+      </c>
+      <c r="M341" t="n">
+        <v>23347.4</v>
+      </c>
+      <c r="N341" t="n">
+        <v>23369.4</v>
+      </c>
+      <c r="O341" t="n">
+        <v>65</v>
+      </c>
+      <c r="P341" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q341" t="n">
+        <v>23359.3</v>
+      </c>
+      <c r="R341" t="n">
+        <v>23292.1</v>
+      </c>
+      <c r="S341" t="n">
+        <v>23363.2</v>
+      </c>
+      <c r="T341" t="n">
+        <v>23195.1</v>
+      </c>
+      <c r="U341" t="n">
+        <v>23279.2</v>
+      </c>
+      <c r="V341" t="n">
+        <v>23273.4</v>
+      </c>
+      <c r="W341" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X341" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y341" t="n">
+        <v>23356</v>
+      </c>
+      <c r="Z341" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="AA341" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB341" t="n">
+        <v>23329.4</v>
+      </c>
+      <c r="AC341" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD341" t="n">
+        <v>23489.4</v>
+      </c>
+      <c r="AE341" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF341" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="AG341" t="inlineStr"/>
+      <c r="AH341" t="inlineStr"/>
+      <c r="AI341" t="inlineStr"/>
+      <c r="AJ341" t="inlineStr"/>
+      <c r="AK341" t="inlineStr"/>
+      <c r="AL341" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-21
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL341"/>
+  <dimension ref="A1:AL343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41468,12 +41468,252 @@
       <c r="AF341" t="n">
         <v>11.4</v>
       </c>
-      <c r="AG341" t="inlineStr"/>
-      <c r="AH341" t="inlineStr"/>
-      <c r="AI341" t="inlineStr"/>
-      <c r="AJ341" t="inlineStr"/>
-      <c r="AK341" t="inlineStr"/>
-      <c r="AL341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>23450</v>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G342" t="n">
+        <v>23437.5</v>
+      </c>
+      <c r="H342" t="n">
+        <v>88</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K342" t="n">
+        <v>7</v>
+      </c>
+      <c r="L342" t="n">
+        <v>23444.1</v>
+      </c>
+      <c r="M342" t="n">
+        <v>23441.8</v>
+      </c>
+      <c r="N342" t="n">
+        <v>23437.5</v>
+      </c>
+      <c r="O342" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="P342" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q342" t="n">
+        <v>23402.9</v>
+      </c>
+      <c r="R342" t="n">
+        <v>23317.2</v>
+      </c>
+      <c r="S342" t="n">
+        <v>23389.2</v>
+      </c>
+      <c r="T342" t="n">
+        <v>23286.8</v>
+      </c>
+      <c r="U342" t="n">
+        <v>23343.6</v>
+      </c>
+      <c r="V342" t="n">
+        <v>23338</v>
+      </c>
+      <c r="W342" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X342" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y342" t="n">
+        <v>23431.4</v>
+      </c>
+      <c r="Z342" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="AA342" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB342" t="n">
+        <v>23397.5</v>
+      </c>
+      <c r="AC342" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD342" t="n">
+        <v>23557.5</v>
+      </c>
+      <c r="AE342" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF342" t="n">
+        <v>11.28</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>74900</v>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G343" t="n">
+        <v>74893.8</v>
+      </c>
+      <c r="H343" t="n">
+        <v>93</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K343" t="n">
+        <v>7</v>
+      </c>
+      <c r="L343" t="n">
+        <v>74922.8</v>
+      </c>
+      <c r="M343" t="n">
+        <v>74913.3</v>
+      </c>
+      <c r="N343" t="n">
+        <v>74891.8</v>
+      </c>
+      <c r="O343" t="n">
+        <v>47</v>
+      </c>
+      <c r="P343" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q343" t="n">
+        <v>74772.10000000001</v>
+      </c>
+      <c r="R343" t="n">
+        <v>74490.60000000001</v>
+      </c>
+      <c r="S343" t="n">
+        <v>74727.5</v>
+      </c>
+      <c r="T343" t="n">
+        <v>73416</v>
+      </c>
+      <c r="U343" t="n">
+        <v>74220.60000000001</v>
+      </c>
+      <c r="V343" t="n">
+        <v>74071.8</v>
+      </c>
+      <c r="W343" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X343" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y343" t="n">
+        <v>74870.2</v>
+      </c>
+      <c r="Z343" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="AA343" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB343" t="n">
+        <v>74693.8</v>
+      </c>
+      <c r="AC343" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD343" t="n">
+        <v>75493.8</v>
+      </c>
+      <c r="AE343" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF343" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AG343" t="inlineStr"/>
+      <c r="AH343" t="inlineStr"/>
+      <c r="AI343" t="inlineStr"/>
+      <c r="AJ343" t="inlineStr"/>
+      <c r="AK343" t="inlineStr"/>
+      <c r="AL343" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-09-24
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL343"/>
+  <dimension ref="A1:AL349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41708,12 +41708,732 @@
       <c r="AF343" t="n">
         <v>11.2</v>
       </c>
-      <c r="AG343" t="inlineStr"/>
-      <c r="AH343" t="inlineStr"/>
-      <c r="AI343" t="inlineStr"/>
-      <c r="AJ343" t="inlineStr"/>
-      <c r="AK343" t="inlineStr"/>
-      <c r="AL343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>73700</v>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G344" t="n">
+        <v>73664.60000000001</v>
+      </c>
+      <c r="H344" t="n">
+        <v>88</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K344" t="n">
+        <v>7</v>
+      </c>
+      <c r="L344" t="n">
+        <v>73707.8</v>
+      </c>
+      <c r="M344" t="n">
+        <v>73819.39999999999</v>
+      </c>
+      <c r="N344" t="n">
+        <v>73670.8</v>
+      </c>
+      <c r="O344" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="P344" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q344" t="n">
+        <v>74360.3</v>
+      </c>
+      <c r="R344" t="n">
+        <v>74164.5</v>
+      </c>
+      <c r="S344" t="n">
+        <v>74973.7</v>
+      </c>
+      <c r="T344" t="n">
+        <v>74604.89999999999</v>
+      </c>
+      <c r="U344" t="n">
+        <v>74815.3</v>
+      </c>
+      <c r="V344" t="n">
+        <v>74789.3</v>
+      </c>
+      <c r="W344" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X344" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y344" t="n">
+        <v>73767.10000000001</v>
+      </c>
+      <c r="Z344" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="AA344" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB344" t="n">
+        <v>73864.60000000001</v>
+      </c>
+      <c r="AC344" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD344" t="n">
+        <v>73064.60000000001</v>
+      </c>
+      <c r="AE344" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF344" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>14:37</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D345" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>55500</v>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G345" t="n">
+        <v>55519.1</v>
+      </c>
+      <c r="H345" t="n">
+        <v>86</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K345" t="n">
+        <v>7</v>
+      </c>
+      <c r="L345" t="n">
+        <v>55459.8</v>
+      </c>
+      <c r="M345" t="n">
+        <v>55491.2</v>
+      </c>
+      <c r="N345" t="n">
+        <v>55497.2</v>
+      </c>
+      <c r="O345" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P345" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q345" t="n">
+        <v>55914.6</v>
+      </c>
+      <c r="R345" t="n">
+        <v>55641.5</v>
+      </c>
+      <c r="S345" t="n">
+        <v>56623.8</v>
+      </c>
+      <c r="T345" t="n">
+        <v>56228.4</v>
+      </c>
+      <c r="U345" t="n">
+        <v>56508</v>
+      </c>
+      <c r="V345" t="n">
+        <v>56426.1</v>
+      </c>
+      <c r="W345" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X345" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y345" t="n">
+        <v>55560.5</v>
+      </c>
+      <c r="Z345" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="AA345" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB345" t="n">
+        <v>55639.1</v>
+      </c>
+      <c r="AC345" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD345" t="n">
+        <v>55159.1</v>
+      </c>
+      <c r="AE345" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF345" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>23100</v>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G346" t="n">
+        <v>23088.7</v>
+      </c>
+      <c r="H346" t="n">
+        <v>98</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K346" t="n">
+        <v>8</v>
+      </c>
+      <c r="L346" t="n">
+        <v>23083.4</v>
+      </c>
+      <c r="M346" t="n">
+        <v>23105.9</v>
+      </c>
+      <c r="N346" t="n">
+        <v>23095.3</v>
+      </c>
+      <c r="O346" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="P346" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q346" t="n">
+        <v>23280.6</v>
+      </c>
+      <c r="R346" t="n">
+        <v>23215.7</v>
+      </c>
+      <c r="S346" t="n">
+        <v>23466.9</v>
+      </c>
+      <c r="T346" t="n">
+        <v>23349.7</v>
+      </c>
+      <c r="U346" t="n">
+        <v>23434</v>
+      </c>
+      <c r="V346" t="n">
+        <v>23408.3</v>
+      </c>
+      <c r="W346" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X346" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y346" t="n">
+        <v>23101.5</v>
+      </c>
+      <c r="Z346" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="AA346" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB346" t="n">
+        <v>23128.7</v>
+      </c>
+      <c r="AC346" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD346" t="n">
+        <v>22968.7</v>
+      </c>
+      <c r="AE346" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF346" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D347" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>55500</v>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G347" t="n">
+        <v>55511.5</v>
+      </c>
+      <c r="H347" t="n">
+        <v>98</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K347" t="n">
+        <v>8</v>
+      </c>
+      <c r="L347" t="n">
+        <v>55476.5</v>
+      </c>
+      <c r="M347" t="n">
+        <v>55496.3</v>
+      </c>
+      <c r="N347" t="n">
+        <v>55531</v>
+      </c>
+      <c r="O347" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="P347" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q347" t="n">
+        <v>55914.6</v>
+      </c>
+      <c r="R347" t="n">
+        <v>55641.5</v>
+      </c>
+      <c r="S347" t="n">
+        <v>56623.8</v>
+      </c>
+      <c r="T347" t="n">
+        <v>56228.4</v>
+      </c>
+      <c r="U347" t="n">
+        <v>56508</v>
+      </c>
+      <c r="V347" t="n">
+        <v>56426.1</v>
+      </c>
+      <c r="W347" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X347" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y347" t="n">
+        <v>55476.8</v>
+      </c>
+      <c r="Z347" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AA347" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB347" t="n">
+        <v>55631.5</v>
+      </c>
+      <c r="AC347" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD347" t="n">
+        <v>55151.5</v>
+      </c>
+      <c r="AE347" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF347" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>73700</v>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G348" t="n">
+        <v>73718</v>
+      </c>
+      <c r="H348" t="n">
+        <v>98</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K348" t="n">
+        <v>8</v>
+      </c>
+      <c r="L348" t="n">
+        <v>73692.60000000001</v>
+      </c>
+      <c r="M348" t="n">
+        <v>73764.3</v>
+      </c>
+      <c r="N348" t="n">
+        <v>73728.89999999999</v>
+      </c>
+      <c r="O348" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="P348" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q348" t="n">
+        <v>74360.3</v>
+      </c>
+      <c r="R348" t="n">
+        <v>74164.5</v>
+      </c>
+      <c r="S348" t="n">
+        <v>74973.7</v>
+      </c>
+      <c r="T348" t="n">
+        <v>74604.89999999999</v>
+      </c>
+      <c r="U348" t="n">
+        <v>74815.3</v>
+      </c>
+      <c r="V348" t="n">
+        <v>74789.3</v>
+      </c>
+      <c r="W348" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X348" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y348" t="n">
+        <v>73752</v>
+      </c>
+      <c r="Z348" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="AA348" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB348" t="n">
+        <v>73918</v>
+      </c>
+      <c r="AC348" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD348" t="n">
+        <v>73118</v>
+      </c>
+      <c r="AE348" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF348" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>23100</v>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G349" t="n">
+        <v>23079.8</v>
+      </c>
+      <c r="H349" t="n">
+        <v>98</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K349" t="n">
+        <v>8</v>
+      </c>
+      <c r="L349" t="n">
+        <v>23091</v>
+      </c>
+      <c r="M349" t="n">
+        <v>23101.4</v>
+      </c>
+      <c r="N349" t="n">
+        <v>23080.5</v>
+      </c>
+      <c r="O349" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="P349" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q349" t="n">
+        <v>23280.6</v>
+      </c>
+      <c r="R349" t="n">
+        <v>23215.7</v>
+      </c>
+      <c r="S349" t="n">
+        <v>23466.9</v>
+      </c>
+      <c r="T349" t="n">
+        <v>23349.7</v>
+      </c>
+      <c r="U349" t="n">
+        <v>23434</v>
+      </c>
+      <c r="V349" t="n">
+        <v>23408.3</v>
+      </c>
+      <c r="W349" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X349" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y349" t="n">
+        <v>23101.5</v>
+      </c>
+      <c r="Z349" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="AA349" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB349" t="n">
+        <v>23119.8</v>
+      </c>
+      <c r="AC349" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD349" t="n">
+        <v>22959.8</v>
+      </c>
+      <c r="AE349" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF349" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="AG349" t="inlineStr"/>
+      <c r="AH349" t="inlineStr"/>
+      <c r="AI349" t="inlineStr"/>
+      <c r="AJ349" t="inlineStr"/>
+      <c r="AK349" t="inlineStr"/>
+      <c r="AL349" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-10-15
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL349"/>
+  <dimension ref="A1:AL351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42428,12 +42428,252 @@
       <c r="AF349" t="n">
         <v>13.1</v>
       </c>
-      <c r="AG349" t="inlineStr"/>
-      <c r="AH349" t="inlineStr"/>
-      <c r="AI349" t="inlineStr"/>
-      <c r="AJ349" t="inlineStr"/>
-      <c r="AK349" t="inlineStr"/>
-      <c r="AL349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>23000</v>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G350" t="n">
+        <v>23017</v>
+      </c>
+      <c r="H350" t="n">
+        <v>80</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K350" t="n">
+        <v>6</v>
+      </c>
+      <c r="L350" t="n">
+        <v>23027.6</v>
+      </c>
+      <c r="M350" t="n">
+        <v>23017.4</v>
+      </c>
+      <c r="N350" t="n">
+        <v>23017</v>
+      </c>
+      <c r="O350" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="P350" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q350" t="n">
+        <v>22752.1</v>
+      </c>
+      <c r="R350" t="n">
+        <v>22637.4</v>
+      </c>
+      <c r="S350" t="n">
+        <v>22757.8</v>
+      </c>
+      <c r="T350" t="n">
+        <v>22558.9</v>
+      </c>
+      <c r="U350" t="n">
+        <v>22658.4</v>
+      </c>
+      <c r="V350" t="n">
+        <v>22634.6</v>
+      </c>
+      <c r="W350" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X350" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y350" t="n">
+        <v>22957.4</v>
+      </c>
+      <c r="Z350" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="AA350" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB350" t="n">
+        <v>22977</v>
+      </c>
+      <c r="AC350" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD350" t="n">
+        <v>23137</v>
+      </c>
+      <c r="AE350" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF350" t="n">
+        <v>14.37</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>74200</v>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G351" t="n">
+        <v>74218.89999999999</v>
+      </c>
+      <c r="H351" t="n">
+        <v>80</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K351" t="n">
+        <v>6</v>
+      </c>
+      <c r="L351" t="n">
+        <v>74237.2</v>
+      </c>
+      <c r="M351" t="n">
+        <v>74178.89999999999</v>
+      </c>
+      <c r="N351" t="n">
+        <v>74218.89999999999</v>
+      </c>
+      <c r="O351" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q351" t="n">
+        <v>73270.5</v>
+      </c>
+      <c r="R351" t="n">
+        <v>72898.7</v>
+      </c>
+      <c r="S351" t="n">
+        <v>73193.89999999999</v>
+      </c>
+      <c r="T351" t="n">
+        <v>72579.3</v>
+      </c>
+      <c r="U351" t="n">
+        <v>72886.60000000001</v>
+      </c>
+      <c r="V351" t="n">
+        <v>72816.8</v>
+      </c>
+      <c r="W351" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X351" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y351" t="n">
+        <v>73991.89999999999</v>
+      </c>
+      <c r="Z351" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="AA351" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB351" t="n">
+        <v>74018.89999999999</v>
+      </c>
+      <c r="AC351" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD351" t="n">
+        <v>74818.89999999999</v>
+      </c>
+      <c r="AE351" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF351" t="n">
+        <v>14.37</v>
+      </c>
+      <c r="AG351" t="inlineStr"/>
+      <c r="AH351" t="inlineStr"/>
+      <c r="AI351" t="inlineStr"/>
+      <c r="AJ351" t="inlineStr"/>
+      <c r="AK351" t="inlineStr"/>
+      <c r="AL351" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-10-19
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL351"/>
+  <dimension ref="A1:AL353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42668,12 +42668,252 @@
       <c r="AF351" t="n">
         <v>14.37</v>
       </c>
-      <c r="AG351" t="inlineStr"/>
-      <c r="AH351" t="inlineStr"/>
-      <c r="AI351" t="inlineStr"/>
-      <c r="AJ351" t="inlineStr"/>
-      <c r="AK351" t="inlineStr"/>
-      <c r="AL351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D352" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>22850</v>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G352" t="n">
+        <v>22859.2</v>
+      </c>
+      <c r="H352" t="n">
+        <v>85</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K352" t="n">
+        <v>6</v>
+      </c>
+      <c r="L352" t="n">
+        <v>22867.8</v>
+      </c>
+      <c r="M352" t="n">
+        <v>22878.8</v>
+      </c>
+      <c r="N352" t="n">
+        <v>22859.9</v>
+      </c>
+      <c r="O352" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="P352" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q352" t="n">
+        <v>23175.1</v>
+      </c>
+      <c r="R352" t="n">
+        <v>22970.8</v>
+      </c>
+      <c r="S352" t="n">
+        <v>23149.8</v>
+      </c>
+      <c r="T352" t="n">
+        <v>22914.3</v>
+      </c>
+      <c r="U352" t="n">
+        <v>23108.1</v>
+      </c>
+      <c r="V352" t="n">
+        <v>23032.1</v>
+      </c>
+      <c r="W352" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X352" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y352" t="n">
+        <v>22923.1</v>
+      </c>
+      <c r="Z352" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="AA352" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB352" t="n">
+        <v>22899.2</v>
+      </c>
+      <c r="AC352" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD352" t="n">
+        <v>22739.2</v>
+      </c>
+      <c r="AE352" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF352" t="n">
+        <v>14.82</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D353" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>73800</v>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G353" t="n">
+        <v>73771</v>
+      </c>
+      <c r="H353" t="n">
+        <v>85</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K353" t="n">
+        <v>6</v>
+      </c>
+      <c r="L353" t="n">
+        <v>73781.39999999999</v>
+      </c>
+      <c r="M353" t="n">
+        <v>73829.39999999999</v>
+      </c>
+      <c r="N353" t="n">
+        <v>73786.7</v>
+      </c>
+      <c r="O353" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="P353" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q353" t="n">
+        <v>74813.10000000001</v>
+      </c>
+      <c r="R353" t="n">
+        <v>74191.3</v>
+      </c>
+      <c r="S353" t="n">
+        <v>74788.8</v>
+      </c>
+      <c r="T353" t="n">
+        <v>74015.7</v>
+      </c>
+      <c r="U353" t="n">
+        <v>74620.3</v>
+      </c>
+      <c r="V353" t="n">
+        <v>74402.2</v>
+      </c>
+      <c r="W353" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X353" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y353" t="n">
+        <v>73971.2</v>
+      </c>
+      <c r="Z353" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="AA353" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB353" t="n">
+        <v>73971</v>
+      </c>
+      <c r="AC353" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD353" t="n">
+        <v>73171</v>
+      </c>
+      <c r="AE353" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF353" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="AG353" t="inlineStr"/>
+      <c r="AH353" t="inlineStr"/>
+      <c r="AI353" t="inlineStr"/>
+      <c r="AJ353" t="inlineStr"/>
+      <c r="AK353" t="inlineStr"/>
+      <c r="AL353" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-10-21
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL353"/>
+  <dimension ref="A1:AL357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42908,12 +42908,492 @@
       <c r="AF353" t="n">
         <v>14.82</v>
       </c>
-      <c r="AG353" t="inlineStr"/>
-      <c r="AH353" t="inlineStr"/>
-      <c r="AI353" t="inlineStr"/>
-      <c r="AJ353" t="inlineStr"/>
-      <c r="AK353" t="inlineStr"/>
-      <c r="AL353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>NIFTY50</t>
+        </is>
+      </c>
+      <c r="D354" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>22700</v>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G354" t="n">
+        <v>22677.4</v>
+      </c>
+      <c r="H354" t="n">
+        <v>85</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K354" t="n">
+        <v>6</v>
+      </c>
+      <c r="L354" t="n">
+        <v>22684.1</v>
+      </c>
+      <c r="M354" t="n">
+        <v>22708.2</v>
+      </c>
+      <c r="N354" t="n">
+        <v>22683.1</v>
+      </c>
+      <c r="O354" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="P354" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q354" t="n">
+        <v>23086.8</v>
+      </c>
+      <c r="R354" t="n">
+        <v>22981.3</v>
+      </c>
+      <c r="S354" t="n">
+        <v>23175.1</v>
+      </c>
+      <c r="T354" t="n">
+        <v>22845.2</v>
+      </c>
+      <c r="U354" t="n">
+        <v>23010.2</v>
+      </c>
+      <c r="V354" t="n">
+        <v>22929.4</v>
+      </c>
+      <c r="W354" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X354" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y354" t="n">
+        <v>22763</v>
+      </c>
+      <c r="Z354" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="AA354" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB354" t="n">
+        <v>22717.4</v>
+      </c>
+      <c r="AC354" t="n">
+        <v>40</v>
+      </c>
+      <c r="AD354" t="n">
+        <v>22557.4</v>
+      </c>
+      <c r="AE354" t="n">
+        <v>120</v>
+      </c>
+      <c r="AF354" t="n">
+        <v>15.89</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D355" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>54800</v>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G355" t="n">
+        <v>54789.8</v>
+      </c>
+      <c r="H355" t="n">
+        <v>95</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K355" t="n">
+        <v>7</v>
+      </c>
+      <c r="L355" t="n">
+        <v>54776.9</v>
+      </c>
+      <c r="M355" t="n">
+        <v>54804.7</v>
+      </c>
+      <c r="N355" t="n">
+        <v>54800.1</v>
+      </c>
+      <c r="O355" t="n">
+        <v>44.7</v>
+      </c>
+      <c r="P355" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q355" t="n">
+        <v>55775</v>
+      </c>
+      <c r="R355" t="n">
+        <v>55595.8</v>
+      </c>
+      <c r="S355" t="n">
+        <v>55882.9</v>
+      </c>
+      <c r="T355" t="n">
+        <v>55335.1</v>
+      </c>
+      <c r="U355" t="n">
+        <v>55609</v>
+      </c>
+      <c r="V355" t="n">
+        <v>55528.4</v>
+      </c>
+      <c r="W355" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X355" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y355" t="n">
+        <v>54951</v>
+      </c>
+      <c r="Z355" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="AA355" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB355" t="n">
+        <v>54909.8</v>
+      </c>
+      <c r="AC355" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD355" t="n">
+        <v>54429.8</v>
+      </c>
+      <c r="AE355" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF355" t="n">
+        <v>15.89</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>73300</v>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G356" t="n">
+        <v>73320.3</v>
+      </c>
+      <c r="H356" t="n">
+        <v>85</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K356" t="n">
+        <v>6</v>
+      </c>
+      <c r="L356" t="n">
+        <v>73332.2</v>
+      </c>
+      <c r="M356" t="n">
+        <v>73405.10000000001</v>
+      </c>
+      <c r="N356" t="n">
+        <v>73334.60000000001</v>
+      </c>
+      <c r="O356" t="n">
+        <v>39</v>
+      </c>
+      <c r="P356" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q356" t="n">
+        <v>74547.2</v>
+      </c>
+      <c r="R356" t="n">
+        <v>74164.7</v>
+      </c>
+      <c r="S356" t="n">
+        <v>74813.10000000001</v>
+      </c>
+      <c r="T356" t="n">
+        <v>73711.10000000001</v>
+      </c>
+      <c r="U356" t="n">
+        <v>74262.10000000001</v>
+      </c>
+      <c r="V356" t="n">
+        <v>73989.3</v>
+      </c>
+      <c r="W356" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X356" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y356" t="n">
+        <v>73562.39999999999</v>
+      </c>
+      <c r="Z356" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AA356" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB356" t="n">
+        <v>73520.3</v>
+      </c>
+      <c r="AC356" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD356" t="n">
+        <v>72720.3</v>
+      </c>
+      <c r="AE356" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF356" t="n">
+        <v>15.85</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D357" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>54800</v>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G357" t="n">
+        <v>54843</v>
+      </c>
+      <c r="H357" t="n">
+        <v>95</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K357" t="n">
+        <v>7</v>
+      </c>
+      <c r="L357" t="n">
+        <v>54799.2</v>
+      </c>
+      <c r="M357" t="n">
+        <v>54803</v>
+      </c>
+      <c r="N357" t="n">
+        <v>54850.6</v>
+      </c>
+      <c r="O357" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="P357" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q357" t="n">
+        <v>55775</v>
+      </c>
+      <c r="R357" t="n">
+        <v>55595.8</v>
+      </c>
+      <c r="S357" t="n">
+        <v>55882.9</v>
+      </c>
+      <c r="T357" t="n">
+        <v>55335.1</v>
+      </c>
+      <c r="U357" t="n">
+        <v>55609</v>
+      </c>
+      <c r="V357" t="n">
+        <v>55528.4</v>
+      </c>
+      <c r="W357" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X357" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y357" t="n">
+        <v>54951</v>
+      </c>
+      <c r="Z357" t="n">
+        <v>0.197</v>
+      </c>
+      <c r="AA357" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB357" t="n">
+        <v>54963</v>
+      </c>
+      <c r="AC357" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD357" t="n">
+        <v>54483</v>
+      </c>
+      <c r="AE357" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF357" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="AG357" t="inlineStr"/>
+      <c r="AH357" t="inlineStr"/>
+      <c r="AI357" t="inlineStr"/>
+      <c r="AJ357" t="inlineStr"/>
+      <c r="AK357" t="inlineStr"/>
+      <c r="AL357" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-10-23
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL357"/>
+  <dimension ref="A1:AL359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43388,12 +43388,252 @@
       <c r="AF357" t="n">
         <v>15.66</v>
       </c>
-      <c r="AG357" t="inlineStr"/>
-      <c r="AH357" t="inlineStr"/>
-      <c r="AI357" t="inlineStr"/>
-      <c r="AJ357" t="inlineStr"/>
-      <c r="AK357" t="inlineStr"/>
-      <c r="AL357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>54000</v>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G358" t="n">
+        <v>54023.1</v>
+      </c>
+      <c r="H358" t="n">
+        <v>95</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K358" t="n">
+        <v>7</v>
+      </c>
+      <c r="L358" t="n">
+        <v>54170.1</v>
+      </c>
+      <c r="M358" t="n">
+        <v>54183.9</v>
+      </c>
+      <c r="N358" t="n">
+        <v>54037.9</v>
+      </c>
+      <c r="O358" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="P358" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q358" t="n">
+        <v>54980.5</v>
+      </c>
+      <c r="R358" t="n">
+        <v>54649.4</v>
+      </c>
+      <c r="S358" t="n">
+        <v>55133.2</v>
+      </c>
+      <c r="T358" t="n">
+        <v>54462.4</v>
+      </c>
+      <c r="U358" t="n">
+        <v>54883.1</v>
+      </c>
+      <c r="V358" t="n">
+        <v>54797.8</v>
+      </c>
+      <c r="W358" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X358" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y358" t="n">
+        <v>54189.1</v>
+      </c>
+      <c r="Z358" t="n">
+        <v>0.307</v>
+      </c>
+      <c r="AA358" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB358" t="n">
+        <v>54143.1</v>
+      </c>
+      <c r="AC358" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD358" t="n">
+        <v>53663.1</v>
+      </c>
+      <c r="AE358" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF358" t="n">
+        <v>16.77</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>54300</v>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="G359" t="n">
+        <v>54287.4</v>
+      </c>
+      <c r="H359" t="n">
+        <v>86</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K359" t="n">
+        <v>7</v>
+      </c>
+      <c r="L359" t="n">
+        <v>54137.4</v>
+      </c>
+      <c r="M359" t="n">
+        <v>54143.1</v>
+      </c>
+      <c r="N359" t="n">
+        <v>54228.8</v>
+      </c>
+      <c r="O359" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="P359" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="Q359" t="n">
+        <v>54980.5</v>
+      </c>
+      <c r="R359" t="n">
+        <v>54649.4</v>
+      </c>
+      <c r="S359" t="n">
+        <v>55133.2</v>
+      </c>
+      <c r="T359" t="n">
+        <v>54462.4</v>
+      </c>
+      <c r="U359" t="n">
+        <v>54883.1</v>
+      </c>
+      <c r="V359" t="n">
+        <v>54797.8</v>
+      </c>
+      <c r="W359" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X359" t="inlineStr">
+        <is>
+          <t>0.382</t>
+        </is>
+      </c>
+      <c r="Y359" t="n">
+        <v>54340.3</v>
+      </c>
+      <c r="Z359" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="AA359" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB359" t="n">
+        <v>54407.4</v>
+      </c>
+      <c r="AC359" t="n">
+        <v>120</v>
+      </c>
+      <c r="AD359" t="n">
+        <v>53927.4</v>
+      </c>
+      <c r="AE359" t="n">
+        <v>360</v>
+      </c>
+      <c r="AF359" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="AG359" t="inlineStr"/>
+      <c r="AH359" t="inlineStr"/>
+      <c r="AI359" t="inlineStr"/>
+      <c r="AJ359" t="inlineStr"/>
+      <c r="AK359" t="inlineStr"/>
+      <c r="AL359" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: nifty precision signals 2026-10-26
</commit_message>
<xml_diff>
--- a/logs/Nifty_Precision_Bot.xlsx
+++ b/logs/Nifty_Precision_Bot.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL359"/>
+  <dimension ref="A1:AL360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43628,12 +43628,132 @@
       <c r="AF359" t="n">
         <v>16.85</v>
       </c>
-      <c r="AG359" t="inlineStr"/>
-      <c r="AH359" t="inlineStr"/>
-      <c r="AI359" t="inlineStr"/>
-      <c r="AJ359" t="inlineStr"/>
-      <c r="AK359" t="inlineStr"/>
-      <c r="AL359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>SENSEX</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>73500</v>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G360" t="n">
+        <v>73457.2</v>
+      </c>
+      <c r="H360" t="n">
+        <v>85</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>ULTRA STRONG</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K360" t="n">
+        <v>6</v>
+      </c>
+      <c r="L360" t="n">
+        <v>73435.89999999999</v>
+      </c>
+      <c r="M360" t="n">
+        <v>73380.8</v>
+      </c>
+      <c r="N360" t="n">
+        <v>73439.39999999999</v>
+      </c>
+      <c r="O360" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="P360" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="Q360" t="n">
+        <v>72979</v>
+      </c>
+      <c r="R360" t="n">
+        <v>72514.60000000001</v>
+      </c>
+      <c r="S360" t="n">
+        <v>73764.5</v>
+      </c>
+      <c r="T360" t="n">
+        <v>72452.60000000001</v>
+      </c>
+      <c r="U360" t="n">
+        <v>73118.7</v>
+      </c>
+      <c r="V360" t="n">
+        <v>73108.60000000001</v>
+      </c>
+      <c r="W360" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X360" t="inlineStr">
+        <is>
+          <t>0.236</t>
+        </is>
+      </c>
+      <c r="Y360" t="n">
+        <v>73272.5</v>
+      </c>
+      <c r="Z360" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="AA360" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AB360" t="n">
+        <v>73257.2</v>
+      </c>
+      <c r="AC360" t="n">
+        <v>200</v>
+      </c>
+      <c r="AD360" t="n">
+        <v>74057.2</v>
+      </c>
+      <c r="AE360" t="n">
+        <v>600</v>
+      </c>
+      <c r="AF360" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="AG360" t="inlineStr"/>
+      <c r="AH360" t="inlineStr"/>
+      <c r="AI360" t="inlineStr"/>
+      <c r="AJ360" t="inlineStr"/>
+      <c r="AK360" t="inlineStr"/>
+      <c r="AL360" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>